<commit_message>
TTA-19：按 AUTOSAR 规则完善浅校验 (#19)
* TTA-19：按 AUTOSAR 规则完善浅校验

System：遵循元模型多重性与 atpSplitable 规则写出拆分片段；Composition 命名空间不区分大小写唯一；System/根原型/ECU/接口 DEST 引用检查；放宽通道与接口映射覆盖校验；新增缺失 TYPE-MAPPING、SYSTEM-VERSION、release 不一致等 WARNING。

SWC：ComSpec 按 SW-IMPL-POLICY 选择；访问类别约束；访问点解析后去重与自动命名避让；CS 对象插入顺序与单项错误隔离；AR-PACKAGE 子元素顺序；公式/控制字符/非 UTF-8/损坏工作簿报错；类型引用元类型检查；大小写唯一；数值上下限比较。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* TTA-19：不匹配 AUTOSAR 版本，规范细则降为 WARNING

删除 arRelease 与输入版本比对；SHORT-NAME 字符集和 128 上限保留（R4.0.3 至 R24-11 一致）；仅大小写不同、访问类别约束、不适用的 ComSpec 列改为 WARNING，交由 EB 等工具链校验；同名与引用错误仍为 ERROR。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* TTA-19：SWC 支持修改单字节编码的 ARXML

片段按目标文件声明的编码写入，无法表示的字符写成字符引用；UTF-16/UTF-32 与 GBK 等多字节编码仍报错。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

---------

Co-authored-by: Tian Yong (uic81119) <uic81119@automotive-wan.com>
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/user/swc/SwcTemplate.xlsx
+++ b/docs/user/swc/SwcTemplate.xlsx
@@ -377,7 +377,7 @@
       <text>
         <t>必填
 默认：—
-数组元素的实现数据类型路径。
+数组元素的实现数据类型路径；引用其他元类（如 SW-BASE-TYPE）报错。
 示例：/Pkg/Types/Mode</t>
       </text>
     </comment>
@@ -477,7 +477,7 @@
       <text>
         <t>必填
 默认：—
-数据元素的实现数据类型路径。
+数据元素的数据类型路径（实现或应用数据类型），DEST 取被引用对象的元类。
 示例：/Pkg/Types/Mode</t>
       </text>
     </comment>
@@ -551,7 +551,7 @@
       <text>
         <t>有参数时必填
 默认：—
-参数的实现数据类型路径；无参数 operation 留空。
+参数的数据类型路径（实现或应用数据类型）；无参数 operation 留空。
 示例：/Pkg/Types/Mode</t>
       </text>
     </comment>
@@ -731,7 +731,7 @@
       <text>
         <t>可选
 默认：N
-Y 时为全部 SR 数据元素创建非队列接收 ComSpec；与正数 Queue Length 互斥。
+Y 时为非队列数据元素创建 NONQUEUED 接收 ComSpec（ENABLE-UPDATE）；全部元素为队列元素时 WARNING 并忽略。
 示例：Y / N</t>
       </text>
     </comment>
@@ -739,7 +739,7 @@
       <text>
         <t>可选
 默认：0 / 不生成
-非负整数；正数生成队列接收 ComSpec；0 或留空不生成，与 Enable Update=Y 互斥。
+非负整数；正数为队列元素（SW-IMPL-POLICY=QUEUED）生成 QUEUED 接收 ComSpec，没有队列元素时 WARNING 并忽略；0 或留空不生成。
 示例：4</t>
       </text>
     </comment>
@@ -765,7 +765,7 @@
       <text>
         <t>必填
 默认：—
-已有 runnable 的简称；须已有对应访问点容器。
+已有或本次 CS P 新建 runnable 的简称；缺少访问点容器时自动创建。
 示例：Run</t>
       </text>
     </comment>
@@ -1372,7 +1372,7 @@
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>名称校验</t>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>新建 Name 和路径各段必须以 ASCII 字母开头，只含字母、数字、下划线，最长 128 字符。枚举 Label 等文本可用中文；Runnable Symbol 使用 C 标识符。自动长名称截断并追加哈希。</t>
+          <t>新建 Name 和路径各段必须以 ASCII 字母开头，只含字母、数字、下划线，最长 128 字符。名称区分大小写；仅大小写不同只 WARNING，按不同对象生成，由 EB 校验。枚举 Label 可用中文，但非 C 标识符会 WARNING（RTE 可能需要 SYMBOL）；Runnable Symbol 使用 C 标识符。自动长名称截断并追加哈希。</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -1500,7 +1500,7 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
     </row>
-    <row r="17" ht="36" customHeight="1">
+    <row r="17" ht="44" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>SR P / SR R</t>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Artifact=Y 时必须指定已有 Runnable Name，且已有对应容器。P：Send（默认）/ Write；R：ReceiveByArgument（默认）/ ReceiveByValue / Read。</t>
+          <t>Artifact=Y 时必须指定已有 Runnable Name，缺少的访问点容器自动创建。P：Send（默认）/ Write；R：ReceiveByArgument（默认）/ ReceiveByValue / Read；队列元素用 ReceiveByValue / Read、Enable Update=Y 时用 Read 只 WARNING，由 EB 校验。</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -1532,7 +1532,7 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>ComSpec 触发</t>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>P：超时非空（含 0）或 E2E=Y。R：Enable Update=Y 或 Queue Length&gt;0，两者互斥。仅填 N 或 Queue Length=0 不触发；新端口为全部数据元素生成。</t>
+          <t>P：超时非空（含 0）或 E2E=Y，按元素 SW-IMPL-POLICY 生成 QUEUED / NONQUEUED 发送 ComSpec。R：Enable Update=Y 作用于非队列元素，Queue Length&gt;0 作用于队列元素，不适用于任何元素时 WARNING 并忽略该列。仅填 N 或 Queue Length=0 不触发。</t>
         </is>
       </c>
       <c r="C19" s="2" t="n"/>
@@ -1548,7 +1548,7 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
           <t>已知限制</t>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>组件及内部行为/访问点容器须按对应功能预先存在；CS 不生成应用错误；SR 接口以外不自动生成数据访问点。无参数 operation 的参数三列全空，不能混用同名有参数声明。</t>
+          <t>组件、内部行为和 PORTS 容器须预先存在，访问点容器自动创建；不支持 PR-Port；CS 不生成应用错误；SR 接口以外不自动生成数据访问点。不接受公式和含换行/制表符的单元格。无参数 operation 的参数三列全空，不能混用同名有参数声明。</t>
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="44" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
           <t>Arrays</t>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>数组元素的实现数据类型路径。</t>
+          <t>数组元素的实现数据类型路径；引用其他元类（如 SW-BASE-TYPE）报错。</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
@@ -2508,7 +2508,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="54" ht="44" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
           <t>SR-Interfaces</t>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>数据元素的实现数据类型路径。</t>
+          <t>数据元素的数据类型路径（实现或应用数据类型），DEST 取被引用对象的元类。</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -2812,7 +2812,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="32" customHeight="1">
+    <row r="64" ht="44" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
         <is>
           <t>CS-Interfaces</t>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>参数的实现数据类型路径；无参数 operation 留空。</t>
+          <t>参数的数据类型路径（实现或应用数据类型）；无参数 operation 留空。</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>Y 时为全部 SR 数据元素创建非队列接收 ComSpec；与正数 Queue Length 互斥。</t>
+          <t>Y 时为非队列数据元素创建 NONQUEUED 接收 ComSpec（ENABLE-UPDATE）；全部元素为队列元素时 WARNING 并忽略。</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>非负整数；正数生成队列接收 ComSpec；0 或留空不生成，与 Enable Update=Y 互斥。</t>
+          <t>非负整数；正数为队列元素（SW-IMPL-POLICY=QUEUED）生成 QUEUED 接收 ComSpec，没有队列元素时 WARNING 并忽略；0 或留空不生成。</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
@@ -3692,7 +3692,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="32" customHeight="1">
+    <row r="93" ht="44" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
           <t>Data Accesses</t>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>已有 runnable 的简称；须已有对应访问点容器。</t>
+          <t>已有或本次 CS P 新建 runnable 的简称；缺少访问点容器时自动创建。</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
@@ -4629,10 +4629,10 @@
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="输入不符合本列规则" error="请按表头批注填写。粘贴可能绕过 Excel 验证，运行工具时仍会完整校验。" promptTitle="填写提示" prompt="可选；默认：ReceiveByArgument。仅 SR 且 Artifact=Y 生效；ReceiveBy* 为显式接收，Read 为隐式读访问。" type="list" errorStyle="stop">
       <formula1>"ReceiveByArgument,ReceiveByValue,Read"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="输入不符合本列规则" error="请按表头批注填写。粘贴可能绕过 Excel 验证，运行工具时仍会完整校验。" promptTitle="填写提示" prompt="可选；默认：N。Y 时为全部 SR 数据元素创建非队列接收 ComSpec；与正数 Queue Length 互斥。" type="list" errorStyle="stop">
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="输入不符合本列规则" error="请按表头批注填写。粘贴可能绕过 Excel 验证，运行工具时仍会完整校验。" promptTitle="填写提示" prompt="可选；默认：N。Y 时为非队列数据元素创建 NONQUEUED 接收 ComSpec（ENABLE-UPDATE）；全部元素为队列元素时 WARNING 并忽略。" type="list" errorStyle="stop">
       <formula1>"Y,N,TRUE,FALSE,YES,NO,1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="输入不符合本列规则" error="请按表头批注填写。粘贴可能绕过 Excel 验证，运行工具时仍会完整校验。" promptTitle="填写提示" prompt="可选；默认：0 / 不生成。非负整数；正数生成队列接收 ComSpec；0 或留空不生成，与 Enable Update=Y 互斥。" type="custom" errorStyle="stop">
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="输入不符合本列规则" error="请按表头批注填写。粘贴可能绕过 Excel 验证，运行工具时仍会完整校验。" promptTitle="填写提示" prompt="可选；默认：0 / 不生成。非负整数；正数为队列元素（SW-IMPL-POLICY=QUEUED）生成 QUEUED 接收 ComSpec，没有队列元素时 WARNING 并忽略；0 或留空不生成。" type="custom" errorStyle="stop">
       <formula1>OR(H2="",IFERROR(AND(MOD(VALUE(H2),1)=0,VALUE(H2)&gt;=0),FALSE))</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>